<commit_message>
Include out-of-period contracts and full Arar value in per-rep totals
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA2XXv3viuKc4AVC546mfn
</commit_message>
<xml_diff>
--- a/إجمالي_مبيعات_المناديب_31-7-2025_إلى_31-7-2026.xlsx
+++ b/إجمالي_مبيعات_المناديب_31-7-2025_إلى_31-7-2026.xlsx
@@ -62,7 +62,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -555,7 +555,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>مبيعات السيارة 6-7 (صافي بعد المرتجع شامل الضريبة)</t>
+          <t>مبيعات السيارة 6-7 (صافي بعد المرتجع)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -588,7 +588,7 @@
         <v/>
       </c>
       <c r="E5" s="4">
-        <f>SUMIFS('مبيعات السيارات 6-7 2026'!J2:J57,'مبيعات السيارات 6-7 2026'!C2:C57,"VHC-1219")</f>
+        <f>SUMIFS('مبيعات السيارات 6-7 2026'!H2:H57,'مبيعات السيارات 6-7 2026'!C2:C57,"VHC-1219")</f>
         <v/>
       </c>
       <c r="F5" s="4">
@@ -620,7 +620,7 @@
         <v/>
       </c>
       <c r="E6" s="4">
-        <f>SUMIFS('مبيعات السيارات 6-7 2026'!J2:J57,'مبيعات السيارات 6-7 2026'!C2:C57,"VHC-3010")</f>
+        <f>SUMIFS('مبيعات السيارات 6-7 2026'!H2:H57,'مبيعات السيارات 6-7 2026'!C2:C57,"VHC-3010")</f>
         <v/>
       </c>
       <c r="F6" s="4">
@@ -698,7 +698,7 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>ملاحظات المراجعة:</t>
+          <t>ملاحظات المراجعة (كل الأرقام بالقيمة الإجمالية كما هي بالمستندات):</t>
         </is>
       </c>
     </row>
@@ -712,7 +712,7 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>2) عصمت: عقدان WHT-2756 و WHT-2758 (16,810.00) موجودان في سجل العقود فقط، بدون فاتورة مبدئية ولا قيد في الكشف – أُضيفا ويحتاجان تأكيد.</t>
+          <t>2) عصمت: عقدان WHT-2756 و WHT-2758 (16,810.00) موجودان في سجل العقود فقط، بدون فاتورة مبدئية ولا قيد في الكشف – تمت إضافتهما.</t>
         </is>
       </c>
     </row>
@@ -726,14 +726,14 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>4) عصمت: WHT-1908 (16,658.75) بتاريخ 30-7-2025 وأبو خالد: WHK-1909 (11,570.00) بتاريخ 30-7-2025 – خارج الفترة بيوم واحد فاستُبعدا (موضحان بالرمادي).</t>
+          <t>4) العقدان WHT-1908 (16,658.75) و WHK-1909 (11,570.00) بتاريخ 30-7-2025 (قبل بداية الفترة بيوم) – أُدرجا بناءً على طلبك.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>5) أبو خالد (WHK): عقد عرعر WHK-2364 أدرجه المحاسب بقيمة العقد كاملة 440,000 بينما المسلّم والمسجل بالكشف 367,803.75 – تم اعتماد المسلّم.</t>
+          <t>5) أبو خالد (WHK): عقد عرعر WHK-2364 أُدرج بالقيمة الكاملة 440,000 بناءً على طلبك، علماً بأن المسجل بكشف الحساب 367,803.75 (الفرق 72,196.25 بدون قيد بالكشف).</t>
         </is>
       </c>
     </row>
@@ -754,26 +754,19 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>8) مبيعات السيارات: السيارة 1219 = عصمت، والسيارة 3010 = عماد. إجمالي المحاسب للسيارة 1219 (38,733.08) لم يخصم 3 فواتير مرتجعة بالكامل (4,123.90) فالصافي 34,609.18.</t>
+          <t>8) مبيعات السيارات: السيارة 1219 = عصمت، والسيارة 3010 = عماد. إجمالي المحاسب للسيارة 1219 (38,733.08) لم يخصم 3 فواتير مرتجعة بالكامل (4,123.90) فالصافي 34,609.18. شيت المرتجعات فيه صفّان مكرران (WS-RET-0002 و 0003).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>9) مبيعات السيارات تشمل ضريبة 15% بينما مبيعات الجملة بدون ضريبة. شيت المرتجعات فيه صفّان مكرران (WS-RET-0002 و 0003).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>10) بعض التواريخ في ملفات المحاسب مقلوبة (يوم/شهر) مثل 2026-11-07 وهي 7-11 أي 11 يوليو – تم تصحيحها.</t>
+          <t>9) بعض التواريخ في ملفات المحاسب مقلوبة (يوم/شهر) مثل 2026-11-07 وهي 7-11 أي 11 يوليو – تم تصحيحها.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="13">
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A1:G1"/>
@@ -781,7 +774,6 @@
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="A18:G18"/>
     <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A20:G20"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A15:G15"/>
@@ -870,11 +862,11 @@
         <v>16658.75</v>
       </c>
       <c r="E2" s="11" t="n">
-        <v>0</v>
+        <v>16658.75</v>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>خارج الفترة</t>
+          <t>صحيح (ملاحظة)</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
@@ -884,7 +876,7 @@
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>تاريخه 2025-07-30 قبل بداية الفترة 31-7-2025</t>
+          <t>تاريخه 2025-07-30 قبل بداية الفترة 31-7-2025 بيوم – أُدرج بناءً على طلبك</t>
         </is>
       </c>
     </row>
@@ -8764,11 +8756,11 @@
         <v>11570</v>
       </c>
       <c r="E2" s="11" t="n">
-        <v>0</v>
+        <v>11570</v>
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>خارج الفترة</t>
+          <t>صحيح (ملاحظة)</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
@@ -8778,7 +8770,7 @@
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>تاريخه 2025-07-30 قبل بداية الفترة 31-7-2025</t>
+          <t>تاريخه 2025-07-30 قبل بداية الفترة 31-7-2025 بيوم – أُدرج بناءً على طلبك</t>
         </is>
       </c>
     </row>
@@ -8903,36 +8895,36 @@
       <c r="H6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n">
+      <c r="A7" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="20" t="n">
+      <c r="B7" s="10" t="n">
         <v>45935</v>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>WHK-2364</t>
         </is>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="11" t="n">
         <v>440000</v>
       </c>
-      <c r="E7" s="21" t="n">
-        <v>367803.75</v>
-      </c>
-      <c r="F7" s="19" t="inlineStr">
-        <is>
-          <t>معدّل</t>
-        </is>
-      </c>
-      <c r="G7" s="19" t="inlineStr">
+      <c r="E7" s="11" t="n">
+        <v>440000</v>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>صحيح (ملاحظة)</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>كشف الحساب</t>
         </is>
       </c>
-      <c r="H7" s="19" t="inlineStr">
-        <is>
-          <t>عقد عرعر: المحاسب أدرج قيمة العقد كاملة 440,000.00، والمسلّم فعلياً حسب كشف الحساب (7 قيود) 367,803.75 – الفرق 72,196.25 بدون مستند تسليم</t>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>عقد عرعر – أُدرج بالقيمة الكاملة 440,000.00 بناءً على طلبك. المسجل بكشف الحساب (7 قيود) 367,803.75 – الفرق 72,196.25 بدون قيد بالكشف</t>
         </is>
       </c>
     </row>
@@ -10202,7 +10194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10210,12 +10202,10 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10246,30 +10236,20 @@
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>قبل الضريبة</t>
+          <t>قيمة الفاتورة</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>الضريبة 15%</t>
+          <t>الحالة</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>الإجمالي</t>
+          <t>الصافي بعد المرتجع</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>الحالة</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>صافي بعد المرتجع</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>الشهر</t>
         </is>
@@ -10300,24 +10280,18 @@
         </is>
       </c>
       <c r="F2" s="4" t="n">
-        <v>296.09</v>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>44.41</v>
+        <v>340.5</v>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H2" s="4" t="n">
         <v>340.5</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J2" s="4" t="n">
-        <v>340.5</v>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -10347,24 +10321,18 @@
         </is>
       </c>
       <c r="F3" s="4" t="n">
-        <v>1856.52</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>278.48</v>
+        <v>2135</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H3" s="4" t="n">
         <v>2135</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="n">
-        <v>2135</v>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -10394,24 +10362,18 @@
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>91.3</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>13.7</v>
+        <v>105</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H4" s="4" t="n">
         <v>105</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>105</v>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -10441,24 +10403,18 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>269.57</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>40.43</v>
+        <v>310</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H5" s="4" t="n">
         <v>310</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>310</v>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -10488,24 +10444,18 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>1745.65</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>261.85</v>
+        <v>2007.5</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H6" s="4" t="n">
         <v>2007.5</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>2007.5</v>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -10535,24 +10485,18 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>1956.52</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>293.48</v>
+        <v>2250</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H7" s="4" t="n">
         <v>2250</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="n">
-        <v>2250</v>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -10582,24 +10526,18 @@
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>1710.43</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>256.57</v>
+        <v>1967</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H8" s="4" t="n">
         <v>1967</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>1967</v>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -10629,24 +10567,18 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>2008.7</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>301.3</v>
+        <v>2310</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H9" s="4" t="n">
         <v>2310</v>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="n">
-        <v>2310</v>
-      </c>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -10676,24 +10608,18 @@
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>828.26</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>124.24</v>
+        <v>952.5</v>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H10" s="4" t="n">
         <v>952.5</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>952.5</v>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -10723,24 +10649,18 @@
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>666.96</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>100.04</v>
+        <v>767</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H11" s="4" t="n">
         <v>767</v>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="n">
-        <v>767</v>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -10770,24 +10690,18 @@
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>1014.78</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>152.22</v>
+        <v>1167</v>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H12" s="4" t="n">
         <v>1167</v>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>1167</v>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -10817,23 +10731,17 @@
         </is>
       </c>
       <c r="F13" s="21" t="n">
-        <v>1468</v>
-      </c>
-      <c r="G13" s="21" t="n">
-        <v>220.2</v>
+        <v>1688.2</v>
+      </c>
+      <c r="G13" s="19" t="inlineStr">
+        <is>
+          <t>مرتجع بالكامل</t>
+        </is>
       </c>
       <c r="H13" s="21" t="n">
-        <v>1688.2</v>
+        <v>0</v>
       </c>
       <c r="I13" s="19" t="inlineStr">
-        <is>
-          <t>مرتجع بالكامل</t>
-        </is>
-      </c>
-      <c r="J13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="19" t="inlineStr">
         <is>
           <t>6-2026</t>
         </is>
@@ -10864,23 +10772,17 @@
         </is>
       </c>
       <c r="F14" s="21" t="n">
-        <v>1468</v>
-      </c>
-      <c r="G14" s="21" t="n">
-        <v>220.2</v>
+        <v>1688.2</v>
+      </c>
+      <c r="G14" s="19" t="inlineStr">
+        <is>
+          <t>مرتجع بالكامل</t>
+        </is>
       </c>
       <c r="H14" s="21" t="n">
-        <v>1688.2</v>
+        <v>0</v>
       </c>
       <c r="I14" s="19" t="inlineStr">
-        <is>
-          <t>مرتجع بالكامل</t>
-        </is>
-      </c>
-      <c r="J14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="19" t="inlineStr">
         <is>
           <t>6-2026</t>
         </is>
@@ -10911,24 +10813,18 @@
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>560.87</v>
-      </c>
-      <c r="G15" s="4" t="n">
-        <v>84.13</v>
+        <v>645</v>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H15" s="4" t="n">
         <v>645</v>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="n">
-        <v>645</v>
-      </c>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -10958,23 +10854,17 @@
         </is>
       </c>
       <c r="F16" s="21" t="n">
-        <v>650</v>
-      </c>
-      <c r="G16" s="21" t="n">
-        <v>97.5</v>
+        <v>747.5</v>
+      </c>
+      <c r="G16" s="19" t="inlineStr">
+        <is>
+          <t>مرتجع بالكامل</t>
+        </is>
       </c>
       <c r="H16" s="21" t="n">
-        <v>747.5</v>
+        <v>0</v>
       </c>
       <c r="I16" s="19" t="inlineStr">
-        <is>
-          <t>مرتجع بالكامل</t>
-        </is>
-      </c>
-      <c r="J16" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="19" t="inlineStr">
         <is>
           <t>6-2026</t>
         </is>
@@ -11005,24 +10895,18 @@
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>1213.04</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>181.96</v>
+        <v>1395</v>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H17" s="4" t="n">
         <v>1395</v>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="n">
-        <v>1395</v>
-      </c>
-      <c r="K17" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -11052,24 +10936,18 @@
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>365.49</v>
-      </c>
-      <c r="G18" s="4" t="n">
-        <v>54.82</v>
+        <v>420.3125</v>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H18" s="4" t="n">
         <v>420.3125</v>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="n">
-        <v>420.3125</v>
-      </c>
-      <c r="K18" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -11099,24 +10977,18 @@
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>222.17</v>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>33.33</v>
+        <v>255.5</v>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H19" s="4" t="n">
         <v>255.5</v>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="n">
-        <v>255.5</v>
-      </c>
-      <c r="K19" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -11146,24 +11018,18 @@
         </is>
       </c>
       <c r="F20" s="4" t="n">
-        <v>647.86</v>
-      </c>
-      <c r="G20" s="4" t="n">
-        <v>97.18000000000001</v>
+        <v>745.04375</v>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H20" s="4" t="n">
         <v>745.04375</v>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J20" s="4" t="n">
-        <v>745.04375</v>
-      </c>
-      <c r="K20" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -11193,24 +11059,18 @@
         </is>
       </c>
       <c r="F21" s="4" t="n">
-        <v>852.83</v>
-      </c>
-      <c r="G21" s="4" t="n">
-        <v>127.92</v>
+        <v>980.75</v>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H21" s="4" t="n">
         <v>980.75</v>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="n">
-        <v>980.75</v>
-      </c>
-      <c r="K21" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -11240,24 +11100,18 @@
         </is>
       </c>
       <c r="F22" s="4" t="n">
-        <v>387.02</v>
-      </c>
-      <c r="G22" s="4" t="n">
-        <v>58.05</v>
+        <v>445.06875</v>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H22" s="4" t="n">
         <v>445.06875</v>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="n">
-        <v>445.06875</v>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -11287,24 +11141,18 @@
         </is>
       </c>
       <c r="F23" s="4" t="n">
-        <v>1356.52</v>
-      </c>
-      <c r="G23" s="4" t="n">
-        <v>203.48</v>
+        <v>1560</v>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H23" s="4" t="n">
         <v>1560</v>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J23" s="4" t="n">
-        <v>1560</v>
-      </c>
-      <c r="K23" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -11334,24 +11182,18 @@
         </is>
       </c>
       <c r="F24" s="4" t="n">
-        <v>993.91</v>
-      </c>
-      <c r="G24" s="4" t="n">
-        <v>149.09</v>
+        <v>1143</v>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H24" s="4" t="n">
         <v>1143</v>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="n">
-        <v>1143</v>
-      </c>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -11381,24 +11223,18 @@
         </is>
       </c>
       <c r="F25" s="4" t="n">
-        <v>539.13</v>
-      </c>
-      <c r="G25" s="4" t="n">
-        <v>80.87</v>
+        <v>620</v>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H25" s="4" t="n">
         <v>620</v>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="n">
-        <v>620</v>
-      </c>
-      <c r="K25" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -11428,24 +11264,18 @@
         </is>
       </c>
       <c r="F26" s="4" t="n">
-        <v>1152.17</v>
-      </c>
-      <c r="G26" s="4" t="n">
-        <v>172.83</v>
+        <v>1325</v>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H26" s="4" t="n">
         <v>1325</v>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J26" s="4" t="n">
-        <v>1325</v>
-      </c>
-      <c r="K26" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -11475,24 +11305,18 @@
         </is>
       </c>
       <c r="F27" s="4" t="n">
-        <v>1082.61</v>
-      </c>
-      <c r="G27" s="4" t="n">
-        <v>162.39</v>
+        <v>1245</v>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H27" s="4" t="n">
         <v>1245</v>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="n">
-        <v>1245</v>
-      </c>
-      <c r="K27" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -11522,24 +11346,18 @@
         </is>
       </c>
       <c r="F28" s="4" t="n">
-        <v>1473.91</v>
-      </c>
-      <c r="G28" s="4" t="n">
-        <v>221.09</v>
+        <v>1695</v>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H28" s="4" t="n">
         <v>1695</v>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="n">
-        <v>1695</v>
-      </c>
-      <c r="K28" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -11569,24 +11387,18 @@
         </is>
       </c>
       <c r="F29" s="4" t="n">
-        <v>130.43</v>
-      </c>
-      <c r="G29" s="4" t="n">
-        <v>19.57</v>
+        <v>150</v>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H29" s="4" t="n">
         <v>150</v>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="n">
-        <v>150</v>
-      </c>
-      <c r="K29" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -11616,24 +11428,18 @@
         </is>
       </c>
       <c r="F30" s="4" t="n">
-        <v>930.4299999999999</v>
-      </c>
-      <c r="G30" s="4" t="n">
-        <v>139.57</v>
+        <v>1070</v>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H30" s="4" t="n">
         <v>1070</v>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J30" s="4" t="n">
-        <v>1070</v>
-      </c>
-      <c r="K30" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -11663,24 +11469,18 @@
         </is>
       </c>
       <c r="F31" s="4" t="n">
-        <v>668.7</v>
-      </c>
-      <c r="G31" s="4" t="n">
-        <v>100.3</v>
+        <v>769</v>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H31" s="4" t="n">
         <v>769</v>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="n">
-        <v>769</v>
-      </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -11710,24 +11510,18 @@
         </is>
       </c>
       <c r="F32" s="4" t="n">
-        <v>139.13</v>
-      </c>
-      <c r="G32" s="4" t="n">
-        <v>20.87</v>
+        <v>160</v>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H32" s="4" t="n">
         <v>160</v>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="n">
-        <v>160</v>
-      </c>
-      <c r="K32" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -11757,24 +11551,18 @@
         </is>
       </c>
       <c r="F33" s="4" t="n">
-        <v>347.83</v>
-      </c>
-      <c r="G33" s="4" t="n">
-        <v>52.17</v>
+        <v>400</v>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H33" s="4" t="n">
         <v>400</v>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="n">
-        <v>400</v>
-      </c>
-      <c r="K33" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -11804,24 +11592,18 @@
         </is>
       </c>
       <c r="F34" s="4" t="n">
-        <v>547.83</v>
-      </c>
-      <c r="G34" s="4" t="n">
-        <v>82.17</v>
+        <v>630</v>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H34" s="4" t="n">
         <v>630</v>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="n">
-        <v>630</v>
-      </c>
-      <c r="K34" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -11851,24 +11633,18 @@
         </is>
       </c>
       <c r="F35" s="4" t="n">
-        <v>513.04</v>
-      </c>
-      <c r="G35" s="4" t="n">
-        <v>76.95999999999999</v>
+        <v>590</v>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H35" s="4" t="n">
         <v>590</v>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="n">
-        <v>590</v>
-      </c>
-      <c r="K35" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -11898,24 +11674,18 @@
         </is>
       </c>
       <c r="F36" s="4" t="n">
-        <v>469.57</v>
-      </c>
-      <c r="G36" s="4" t="n">
-        <v>70.43000000000001</v>
+        <v>540</v>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H36" s="4" t="n">
         <v>540</v>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J36" s="4" t="n">
-        <v>540</v>
-      </c>
-      <c r="K36" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -11945,24 +11715,18 @@
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>260.87</v>
-      </c>
-      <c r="G37" s="4" t="n">
-        <v>39.13</v>
+        <v>300</v>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H37" s="4" t="n">
         <v>300</v>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J37" s="4" t="n">
-        <v>300</v>
-      </c>
-      <c r="K37" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -11992,24 +11756,18 @@
         </is>
       </c>
       <c r="F38" s="4" t="n">
-        <v>734.78</v>
-      </c>
-      <c r="G38" s="4" t="n">
-        <v>110.22</v>
+        <v>845</v>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H38" s="4" t="n">
         <v>845</v>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J38" s="4" t="n">
-        <v>845</v>
-      </c>
-      <c r="K38" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12039,24 +11797,18 @@
         </is>
       </c>
       <c r="F39" s="4" t="n">
-        <v>277.39</v>
-      </c>
-      <c r="G39" s="4" t="n">
-        <v>41.61</v>
+        <v>319</v>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H39" s="4" t="n">
         <v>319</v>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J39" s="4" t="n">
-        <v>319</v>
-      </c>
-      <c r="K39" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12086,24 +11838,18 @@
         </is>
       </c>
       <c r="F40" s="4" t="n">
-        <v>572.17</v>
-      </c>
-      <c r="G40" s="4" t="n">
-        <v>85.83</v>
+        <v>658</v>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H40" s="4" t="n">
         <v>658</v>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J40" s="4" t="n">
-        <v>658</v>
-      </c>
-      <c r="K40" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12133,24 +11879,18 @@
         </is>
       </c>
       <c r="F41" s="4" t="n">
-        <v>240.87</v>
-      </c>
-      <c r="G41" s="4" t="n">
-        <v>36.13</v>
+        <v>277</v>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H41" s="4" t="n">
         <v>277</v>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="n">
-        <v>277</v>
-      </c>
-      <c r="K41" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12180,24 +11920,18 @@
         </is>
       </c>
       <c r="F42" s="4" t="n">
-        <v>195.65</v>
-      </c>
-      <c r="G42" s="4" t="n">
-        <v>29.35</v>
+        <v>225</v>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H42" s="4" t="n">
         <v>225</v>
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J42" s="4" t="n">
-        <v>225</v>
-      </c>
-      <c r="K42" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12227,24 +11961,18 @@
         </is>
       </c>
       <c r="F43" s="4" t="n">
-        <v>382.61</v>
-      </c>
-      <c r="G43" s="4" t="n">
-        <v>57.39</v>
+        <v>440</v>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H43" s="4" t="n">
         <v>440</v>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J43" s="4" t="n">
-        <v>440</v>
-      </c>
-      <c r="K43" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12274,24 +12002,18 @@
         </is>
       </c>
       <c r="F44" s="4" t="n">
-        <v>391.3</v>
-      </c>
-      <c r="G44" s="4" t="n">
-        <v>58.7</v>
+        <v>450</v>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H44" s="4" t="n">
         <v>450</v>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J44" s="4" t="n">
-        <v>450</v>
-      </c>
-      <c r="K44" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12321,24 +12043,18 @@
         </is>
       </c>
       <c r="F45" s="4" t="n">
-        <v>1786.74</v>
-      </c>
-      <c r="G45" s="4" t="n">
-        <v>268.01</v>
+        <v>2054.75</v>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H45" s="4" t="n">
         <v>2054.75</v>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J45" s="4" t="n">
-        <v>2054.75</v>
-      </c>
-      <c r="K45" s="3" t="inlineStr">
-        <is>
           <t>6-2026</t>
         </is>
       </c>
@@ -12368,24 +12084,18 @@
         </is>
       </c>
       <c r="F46" s="4" t="n">
-        <v>1560.87</v>
-      </c>
-      <c r="G46" s="4" t="n">
-        <v>234.13</v>
+        <v>1795</v>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H46" s="4" t="n">
         <v>1795</v>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J46" s="4" t="n">
-        <v>1795</v>
-      </c>
-      <c r="K46" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12415,24 +12125,18 @@
         </is>
       </c>
       <c r="F47" s="4" t="n">
-        <v>647.83</v>
-      </c>
-      <c r="G47" s="4" t="n">
-        <v>97.17</v>
+        <v>745</v>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H47" s="4" t="n">
         <v>745</v>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J47" s="4" t="n">
-        <v>745</v>
-      </c>
-      <c r="K47" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12462,24 +12166,18 @@
         </is>
       </c>
       <c r="F48" s="4" t="n">
-        <v>256.52</v>
-      </c>
-      <c r="G48" s="4" t="n">
-        <v>38.48</v>
+        <v>295</v>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H48" s="4" t="n">
         <v>295</v>
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J48" s="4" t="n">
-        <v>295</v>
-      </c>
-      <c r="K48" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12509,24 +12207,18 @@
         </is>
       </c>
       <c r="F49" s="4" t="n">
-        <v>247.83</v>
-      </c>
-      <c r="G49" s="4" t="n">
-        <v>37.17</v>
+        <v>285</v>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H49" s="4" t="n">
         <v>285</v>
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J49" s="4" t="n">
-        <v>285</v>
-      </c>
-      <c r="K49" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12556,24 +12248,18 @@
         </is>
       </c>
       <c r="F50" s="4" t="n">
-        <v>126.09</v>
-      </c>
-      <c r="G50" s="4" t="n">
-        <v>18.91</v>
+        <v>145</v>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H50" s="4" t="n">
         <v>145</v>
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J50" s="4" t="n">
-        <v>145</v>
-      </c>
-      <c r="K50" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12603,24 +12289,18 @@
         </is>
       </c>
       <c r="F51" s="4" t="n">
-        <v>234.78</v>
-      </c>
-      <c r="G51" s="4" t="n">
-        <v>35.22</v>
+        <v>270</v>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H51" s="4" t="n">
         <v>270</v>
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J51" s="4" t="n">
-        <v>270</v>
-      </c>
-      <c r="K51" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12650,24 +12330,18 @@
         </is>
       </c>
       <c r="F52" s="4" t="n">
-        <v>130.43</v>
-      </c>
-      <c r="G52" s="4" t="n">
-        <v>19.57</v>
+        <v>150</v>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H52" s="4" t="n">
         <v>150</v>
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J52" s="4" t="n">
-        <v>150</v>
-      </c>
-      <c r="K52" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12697,24 +12371,18 @@
         </is>
       </c>
       <c r="F53" s="4" t="n">
-        <v>108.7</v>
-      </c>
-      <c r="G53" s="4" t="n">
-        <v>16.3</v>
+        <v>125</v>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H53" s="4" t="n">
         <v>125</v>
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J53" s="4" t="n">
-        <v>125</v>
-      </c>
-      <c r="K53" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12744,24 +12412,18 @@
         </is>
       </c>
       <c r="F54" s="4" t="n">
-        <v>108.7</v>
-      </c>
-      <c r="G54" s="4" t="n">
-        <v>16.3</v>
+        <v>125</v>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H54" s="4" t="n">
         <v>125</v>
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J54" s="4" t="n">
-        <v>125</v>
-      </c>
-      <c r="K54" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12791,24 +12453,18 @@
         </is>
       </c>
       <c r="F55" s="4" t="n">
-        <v>234.78</v>
-      </c>
-      <c r="G55" s="4" t="n">
-        <v>35.22</v>
+        <v>270</v>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H55" s="4" t="n">
         <v>270</v>
       </c>
       <c r="I55" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J55" s="4" t="n">
-        <v>270</v>
-      </c>
-      <c r="K55" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12838,24 +12494,18 @@
         </is>
       </c>
       <c r="F56" s="4" t="n">
-        <v>108.7</v>
-      </c>
-      <c r="G56" s="4" t="n">
-        <v>16.3</v>
+        <v>125</v>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H56" s="4" t="n">
         <v>125</v>
       </c>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J56" s="4" t="n">
-        <v>125</v>
-      </c>
-      <c r="K56" s="3" t="inlineStr">
-        <is>
           <t>7-2026</t>
         </is>
       </c>
@@ -12885,23 +12535,17 @@
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>65.22</v>
-      </c>
-      <c r="G57" s="4" t="n">
-        <v>9.779999999999999</v>
+        <v>75</v>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>مكتمل</t>
+        </is>
       </c>
       <c r="H57" s="4" t="n">
         <v>75</v>
       </c>
       <c r="I57" s="3" t="inlineStr">
-        <is>
-          <t>مكتمل</t>
-        </is>
-      </c>
-      <c r="J57" s="4" t="n">
-        <v>75</v>
-      </c>
-      <c r="K57" s="3" t="inlineStr">
         <is>
           <t>7-2026</t>
         </is>
@@ -12921,20 +12565,12 @@
         <f>SUM(F2:F57)</f>
         <v/>
       </c>
-      <c r="G58" s="6">
-        <f>SUM(G2:G57)</f>
-        <v/>
-      </c>
+      <c r="G58" s="5" t="inlineStr"/>
       <c r="H58" s="6">
         <f>SUM(H2:H57)</f>
         <v/>
       </c>
-      <c r="I58" s="5" t="inlineStr"/>
-      <c r="J58" s="6">
-        <f>SUM(J2:J57)</f>
-        <v/>
-      </c>
-      <c r="K58" s="5" t="n"/>
+      <c r="I58" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>